<commit_message>
lesson16 database - 24.10.2025
</commit_message>
<xml_diff>
--- a/1. Database Design/Java24 QuyenPhan Database Design.xlsx
+++ b/1. Database Design/Java24 QuyenPhan Database Design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java24\3. Database\1. Database Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E3DC602-657D-4999-9A90-0C60DE39EE9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D6F90C-AF3E-4FED-A40B-FF5280567487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1860" windowWidth="38640" windowHeight="21120" tabRatio="433" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1502,7 +1502,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D189" authorId="2" shapeId="0" xr:uid="{9BDC8936-92C9-43A1-9379-AB9B7024CE45}">
+    <comment ref="D188" authorId="2" shapeId="0" xr:uid="{9BDC8936-92C9-43A1-9379-AB9B7024CE45}">
       <text>
         <r>
           <rPr>
@@ -1526,7 +1526,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G189" authorId="2" shapeId="0" xr:uid="{6AE8310D-3BF7-4201-92B2-A2B94D757B52}">
+    <comment ref="G188" authorId="2" shapeId="0" xr:uid="{6AE8310D-3BF7-4201-92B2-A2B94D757B52}">
       <text>
         <r>
           <rPr>
@@ -1550,7 +1550,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D203" authorId="2" shapeId="0" xr:uid="{9B933F05-4824-40FF-A0CC-44296B8D3399}">
+    <comment ref="D202" authorId="2" shapeId="0" xr:uid="{9B933F05-4824-40FF-A0CC-44296B8D3399}">
       <text>
         <r>
           <rPr>
@@ -1574,7 +1574,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G203" authorId="2" shapeId="0" xr:uid="{A1ACCF64-494E-4A04-BC4E-BB52726C36B4}">
+    <comment ref="G202" authorId="2" shapeId="0" xr:uid="{A1ACCF64-494E-4A04-BC4E-BB52726C36B4}">
       <text>
         <r>
           <rPr>
@@ -1598,7 +1598,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C224" authorId="2" shapeId="0" xr:uid="{650603E4-1922-4F3D-BF57-A44480C7E756}">
+    <comment ref="C223" authorId="2" shapeId="0" xr:uid="{650603E4-1922-4F3D-BF57-A44480C7E756}">
       <text>
         <r>
           <rPr>
@@ -1612,7 +1612,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D224" authorId="2" shapeId="0" xr:uid="{23A98BCD-8F58-45E6-803E-7B59DCF7EE56}">
+    <comment ref="D223" authorId="2" shapeId="0" xr:uid="{23A98BCD-8F58-45E6-803E-7B59DCF7EE56}">
       <text>
         <r>
           <rPr>
@@ -1636,7 +1636,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E224" authorId="2" shapeId="0" xr:uid="{2B9AFA3A-E429-42C7-BCF0-DD3595633DCF}">
+    <comment ref="E223" authorId="2" shapeId="0" xr:uid="{2B9AFA3A-E429-42C7-BCF0-DD3595633DCF}">
       <text>
         <r>
           <rPr>
@@ -1660,7 +1660,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G224" authorId="2" shapeId="0" xr:uid="{90AC3731-A473-470A-BB5D-0A799C6457A9}">
+    <comment ref="G223" authorId="2" shapeId="0" xr:uid="{90AC3731-A473-470A-BB5D-0A799C6457A9}">
       <text>
         <r>
           <rPr>
@@ -3392,9 +3392,6 @@
     <t>T18 10 Địa Chỉ</t>
   </si>
   <si>
-    <t>T16 5 Nhân Viên</t>
-  </si>
-  <si>
     <t>T19</t>
   </si>
   <si>
@@ -3404,9 +3401,6 @@
     <t>Ví điện tử</t>
   </si>
   <si>
-    <t>Quan trọng, cần có dữ liệu chính xác để demo nhiều trường hợp</t>
-  </si>
-  <si>
     <t>Chờ xác nhận</t>
   </si>
   <si>
@@ -3458,9 +3452,6 @@
     <t>Nhân Viên 5</t>
   </si>
   <si>
-    <t>Lê Tèo</t>
-  </si>
-  <si>
     <t>c1@gmal.com</t>
   </si>
   <si>
@@ -3470,79 +3461,52 @@
     <t>$2a$12$w0bs0MW/O3nTyMhuv0r1jOjq2gOaxLxkZgms7u/khHRmtCh3S/Hpu</t>
   </si>
   <si>
-    <t>Văn An</t>
-  </si>
-  <si>
     <t>c2@gmal.com</t>
   </si>
   <si>
     <t>c2auto</t>
   </si>
   <si>
-    <t>Nguyễn A</t>
-  </si>
-  <si>
     <t>c3@gmal.com</t>
   </si>
   <si>
     <t>c3def</t>
   </si>
   <si>
-    <t>Phan Tuấn</t>
-  </si>
-  <si>
     <t>c4@gmal.com</t>
   </si>
   <si>
     <t>c4auto</t>
   </si>
   <si>
-    <t>Hoàng Tiên</t>
-  </si>
-  <si>
     <t>c5@gmal.com</t>
   </si>
   <si>
     <t>c5def</t>
   </si>
   <si>
-    <t>Phạm Ngọc</t>
-  </si>
-  <si>
     <t>c6@gmal.com</t>
   </si>
   <si>
     <t>c6auto</t>
   </si>
   <si>
-    <t>Đoạn Tú</t>
-  </si>
-  <si>
     <t>c7@gmal.com</t>
   </si>
   <si>
     <t>c7def</t>
   </si>
   <si>
-    <t>Hoàng B</t>
-  </si>
-  <si>
     <t>c8@gmal.com</t>
   </si>
   <si>
     <t>c8auto</t>
   </si>
   <si>
-    <t>Lê Huân</t>
-  </si>
-  <si>
     <t>c9@gmal.com</t>
   </si>
   <si>
     <t>c9def</t>
-  </si>
-  <si>
-    <t>Nam Ban</t>
   </si>
   <si>
     <t>c10@gmal.com</t>
@@ -3726,6 +3690,42 @@
   </si>
   <si>
     <t>Role 5</t>
+  </si>
+  <si>
+    <t>Khách hàng 1</t>
+  </si>
+  <si>
+    <t>Khách hàng 2</t>
+  </si>
+  <si>
+    <t>Khách hàng 3</t>
+  </si>
+  <si>
+    <t>Khách hàng 4</t>
+  </si>
+  <si>
+    <t>Khách hàng 5</t>
+  </si>
+  <si>
+    <t>Khách hàng 6</t>
+  </si>
+  <si>
+    <t>Khách hàng 7</t>
+  </si>
+  <si>
+    <t>Khách hàng 8</t>
+  </si>
+  <si>
+    <t>Khách hàng 9</t>
+  </si>
+  <si>
+    <t>Khách hàng 10</t>
+  </si>
+  <si>
+    <t>T16 10 Nhân Viên</t>
+  </si>
+  <si>
+    <t>C12_ITEM_DETAIL_ID</t>
   </si>
 </sst>
 </file>
@@ -4007,7 +4007,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -4063,43 +4063,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -4114,7 +4077,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4291,7 +4254,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4309,32 +4272,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -4346,13 +4291,19 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -9133,7 +9084,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19C125E9-733D-4F85-B782-7EFA49F565B4}">
-  <dimension ref="A1:K1000"/>
+  <dimension ref="A1:K999"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="49" customWidth="1"/>
@@ -9150,14 +9101,14 @@
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="49" t="s">
-        <v>534</v>
+        <v>522</v>
       </c>
       <c r="B2" s="63" t="s">
         <v>215</v>
       </c>
       <c r="C2" s="49"/>
       <c r="D2" s="49" t="s">
-        <v>533</v>
+        <v>521</v>
       </c>
       <c r="E2" s="49"/>
     </row>
@@ -9459,7 +9410,7 @@
     <row r="25" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="49" t="s">
-        <v>536</v>
+        <v>524</v>
       </c>
       <c r="B26" s="63" t="s">
         <v>218</v>
@@ -9626,16 +9577,16 @@
     <row r="39" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="49" t="s">
-        <v>535</v>
+        <v>523</v>
       </c>
       <c r="B40" s="62" t="s">
         <v>222</v>
       </c>
       <c r="C40" s="49" t="s">
-        <v>537</v>
+        <v>525</v>
       </c>
       <c r="D40" s="49" t="s">
-        <v>538</v>
+        <v>526</v>
       </c>
       <c r="E40" s="49"/>
       <c r="F40" s="49"/>
@@ -9673,54 +9624,54 @@
       <c r="C43" s="72" t="s">
         <v>422</v>
       </c>
-      <c r="D43" s="71"/>
-      <c r="E43" s="71"/>
-      <c r="F43" s="71"/>
+      <c r="D43" s="73"/>
+      <c r="E43" s="73"/>
+      <c r="F43" s="73"/>
       <c r="G43" s="49"/>
     </row>
     <row r="44" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="49"/>
-      <c r="C44" s="71"/>
-      <c r="D44" s="71"/>
-      <c r="E44" s="71"/>
-      <c r="F44" s="71"/>
+      <c r="C44" s="73"/>
+      <c r="D44" s="73"/>
+      <c r="E44" s="73"/>
+      <c r="F44" s="73"/>
       <c r="G44" s="49"/>
     </row>
     <row r="45" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="49"/>
-      <c r="C45" s="71"/>
-      <c r="D45" s="71"/>
-      <c r="E45" s="71"/>
-      <c r="F45" s="71"/>
+      <c r="C45" s="73"/>
+      <c r="D45" s="73"/>
+      <c r="E45" s="73"/>
+      <c r="F45" s="73"/>
       <c r="G45" s="49"/>
     </row>
     <row r="46" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="49"/>
-      <c r="C46" s="71"/>
-      <c r="D46" s="71"/>
-      <c r="E46" s="71"/>
-      <c r="F46" s="71"/>
+      <c r="C46" s="73"/>
+      <c r="D46" s="73"/>
+      <c r="E46" s="73"/>
+      <c r="F46" s="73"/>
       <c r="G46" s="49"/>
     </row>
     <row r="47" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D47" s="44" t="s">
-        <v>539</v>
+        <v>527</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D48" s="55" t="s">
-        <v>540</v>
+        <v>528</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="49" t="s">
-        <v>535</v>
+        <v>523</v>
       </c>
       <c r="B49" s="62" t="s">
         <v>241</v>
       </c>
       <c r="D49" t="s">
-        <v>545</v>
+        <v>533</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -9738,7 +9689,7 @@
       <c r="B51" s="2">
         <v>1</v>
       </c>
-      <c r="C51" s="73" t="s">
+      <c r="C51" s="74" t="s">
         <v>425</v>
       </c>
       <c r="D51" s="2">
@@ -9749,7 +9700,7 @@
       <c r="B52" s="2">
         <v>2</v>
       </c>
-      <c r="C52" s="73"/>
+      <c r="C52" s="74"/>
       <c r="D52" s="2">
         <v>2</v>
       </c>
@@ -9758,7 +9709,7 @@
       <c r="B53" s="2">
         <v>3</v>
       </c>
-      <c r="C53" s="73"/>
+      <c r="C53" s="74"/>
       <c r="D53" s="2">
         <v>3</v>
       </c>
@@ -9767,7 +9718,7 @@
       <c r="B54" s="2">
         <v>4</v>
       </c>
-      <c r="C54" s="73"/>
+      <c r="C54" s="74"/>
       <c r="D54" s="2">
         <v>4</v>
       </c>
@@ -9776,7 +9727,7 @@
       <c r="B55" s="2">
         <v>5</v>
       </c>
-      <c r="C55" s="73"/>
+      <c r="C55" s="74"/>
       <c r="D55" s="2">
         <v>5</v>
       </c>
@@ -9785,7 +9736,7 @@
       <c r="B56" s="2">
         <v>6</v>
       </c>
-      <c r="C56" s="73"/>
+      <c r="C56" s="74"/>
       <c r="D56" s="2">
         <v>6</v>
       </c>
@@ -9794,7 +9745,7 @@
       <c r="B57" s="2">
         <v>7</v>
       </c>
-      <c r="C57" s="73"/>
+      <c r="C57" s="74"/>
       <c r="D57" s="2">
         <v>7</v>
       </c>
@@ -9803,7 +9754,7 @@
       <c r="B58" s="2">
         <v>8</v>
       </c>
-      <c r="C58" s="73"/>
+      <c r="C58" s="74"/>
       <c r="D58" s="2">
         <v>8</v>
       </c>
@@ -9812,7 +9763,7 @@
       <c r="B59" s="2">
         <v>9</v>
       </c>
-      <c r="C59" s="73"/>
+      <c r="C59" s="74"/>
       <c r="D59" s="2">
         <v>9</v>
       </c>
@@ -9821,7 +9772,7 @@
       <c r="B60" s="2">
         <v>10</v>
       </c>
-      <c r="C60" s="73"/>
+      <c r="C60" s="74"/>
       <c r="D60" s="2">
         <v>10</v>
       </c>
@@ -9830,16 +9781,16 @@
     <row r="62" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="63" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="49" t="s">
-        <v>535</v>
+        <v>523</v>
       </c>
       <c r="B63" s="62" t="s">
         <v>248</v>
       </c>
       <c r="C63" s="49" t="s">
-        <v>543</v>
+        <v>531</v>
       </c>
       <c r="F63" s="49" t="s">
-        <v>542</v>
+        <v>530</v>
       </c>
     </row>
     <row r="64" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -9863,35 +9814,35 @@
       <c r="B65" s="49" t="s">
         <v>421</v>
       </c>
-      <c r="C65" s="69" t="s">
-        <v>541</v>
-      </c>
-      <c r="D65" s="70"/>
-      <c r="E65" s="70"/>
-      <c r="F65" s="70"/>
+      <c r="C65" s="75" t="s">
+        <v>529</v>
+      </c>
+      <c r="D65" s="76"/>
+      <c r="E65" s="76"/>
+      <c r="F65" s="76"/>
     </row>
     <row r="66" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C66" s="71"/>
-      <c r="D66" s="71"/>
-      <c r="E66" s="71"/>
-      <c r="F66" s="71"/>
+      <c r="C66" s="73"/>
+      <c r="D66" s="73"/>
+      <c r="E66" s="73"/>
+      <c r="F66" s="73"/>
     </row>
     <row r="67" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C67" s="71"/>
-      <c r="D67" s="71"/>
-      <c r="E67" s="71"/>
-      <c r="F67" s="71"/>
+      <c r="C67" s="73"/>
+      <c r="D67" s="73"/>
+      <c r="E67" s="73"/>
+      <c r="F67" s="73"/>
     </row>
     <row r="68" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C68" s="71"/>
-      <c r="D68" s="71"/>
-      <c r="E68" s="71"/>
-      <c r="F68" s="71"/>
+      <c r="C68" s="73"/>
+      <c r="D68" s="73"/>
+      <c r="E68" s="73"/>
+      <c r="F68" s="73"/>
     </row>
     <row r="69" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="70" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
-        <v>534</v>
+        <v>522</v>
       </c>
       <c r="B70" s="62" t="s">
         <v>254</v>
@@ -9967,7 +9918,7 @@
     <row r="78" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="79" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="49" t="s">
-        <v>534</v>
+        <v>522</v>
       </c>
       <c r="B79" s="62" t="s">
         <v>260</v>
@@ -9985,7 +9936,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="2">
         <v>1</v>
       </c>
@@ -9996,7 +9947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B82" s="2">
         <v>2</v>
       </c>
@@ -10007,7 +9958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B83" s="2">
         <v>3</v>
       </c>
@@ -10018,7 +9969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B84" s="2">
         <v>4</v>
       </c>
@@ -10029,7 +9980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B85" s="2">
         <v>5</v>
       </c>
@@ -10040,7 +9991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B86" s="2">
         <v>6</v>
       </c>
@@ -10051,7 +10002,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="2">
         <v>7</v>
       </c>
@@ -10062,17 +10013,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="49" t="s">
-        <v>535</v>
-      </c>
-      <c r="B90" s="48" t="s">
+        <v>523</v>
+      </c>
+      <c r="B90" s="62" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="91" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B91" s="11" t="s">
         <v>268</v>
       </c>
@@ -10080,40 +10031,41 @@
         <v>267</v>
       </c>
     </row>
-    <row r="92" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B92" s="69" t="s">
+    <row r="92" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B92" s="75" t="s">
         <v>436</v>
       </c>
-      <c r="C92" s="70"/>
-    </row>
-    <row r="93" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B93" s="71"/>
-      <c r="C93" s="71"/>
-    </row>
-    <row r="94" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B94" s="71"/>
-      <c r="C94" s="71"/>
-    </row>
-    <row r="95" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="C92" s="76"/>
+    </row>
+    <row r="93" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B93" s="73"/>
+      <c r="C93" s="73"/>
+    </row>
+    <row r="94" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B94" s="73"/>
+      <c r="C94" s="73"/>
+    </row>
+    <row r="95" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D96" s="49" t="s">
+        <v>537</v>
+      </c>
+      <c r="E96" s="49" t="s">
+        <v>455</v>
+      </c>
+      <c r="F96" s="49" t="s">
+        <v>456</v>
+      </c>
+      <c r="G96" s="49" t="s">
+        <v>559</v>
+      </c>
+    </row>
     <row r="97" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="49" t="s">
-        <v>534</v>
-      </c>
-      <c r="B97" s="48" t="s">
+        <v>522</v>
+      </c>
+      <c r="B97" s="62" t="s">
         <v>275</v>
-      </c>
-      <c r="D97" s="49" t="s">
-        <v>549</v>
-      </c>
-      <c r="E97" s="49" t="s">
-        <v>455</v>
-      </c>
-      <c r="F97" s="49" t="s">
-        <v>456</v>
-      </c>
-      <c r="G97" s="49" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10152,7 +10104,7 @@
       <c r="F99" s="52">
         <v>1</v>
       </c>
-      <c r="G99" s="74">
+      <c r="G99" s="52">
         <v>1</v>
       </c>
     </row>
@@ -10164,7 +10116,7 @@
         <v>439</v>
       </c>
       <c r="D100" s="52">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E100" s="52">
         <v>2</v>
@@ -10172,7 +10124,7 @@
       <c r="F100" s="52">
         <v>2</v>
       </c>
-      <c r="G100" s="74">
+      <c r="G100" s="52">
         <v>2</v>
       </c>
     </row>
@@ -10184,7 +10136,7 @@
         <v>441</v>
       </c>
       <c r="D101" s="52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E101" s="52">
         <v>3</v>
@@ -10192,7 +10144,7 @@
       <c r="F101" s="52">
         <v>3</v>
       </c>
-      <c r="G101" s="74">
+      <c r="G101" s="52">
         <v>3</v>
       </c>
     </row>
@@ -10204,7 +10156,7 @@
         <v>443</v>
       </c>
       <c r="D102" s="52">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E102" s="52">
         <v>4</v>
@@ -10212,7 +10164,7 @@
       <c r="F102" s="52">
         <v>4</v>
       </c>
-      <c r="G102" s="74">
+      <c r="G102" s="52">
         <v>4</v>
       </c>
     </row>
@@ -10224,7 +10176,7 @@
         <v>445</v>
       </c>
       <c r="D103" s="52">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E103" s="52">
         <v>5</v>
@@ -10232,7 +10184,7 @@
       <c r="F103" s="52">
         <v>5</v>
       </c>
-      <c r="G103" s="74">
+      <c r="G103" s="52">
         <v>5</v>
       </c>
     </row>
@@ -10244,7 +10196,7 @@
         <v>439</v>
       </c>
       <c r="D104" s="52">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E104" s="52">
         <v>6</v>
@@ -10252,7 +10204,7 @@
       <c r="F104" s="52">
         <v>6</v>
       </c>
-      <c r="G104" s="74">
+      <c r="G104" s="52">
         <v>8</v>
       </c>
     </row>
@@ -10264,7 +10216,7 @@
         <v>441</v>
       </c>
       <c r="D105" s="52">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E105" s="52">
         <v>7</v>
@@ -10272,7 +10224,7 @@
       <c r="F105" s="52">
         <v>7</v>
       </c>
-      <c r="G105" s="74">
+      <c r="G105" s="52">
         <v>7</v>
       </c>
     </row>
@@ -10284,7 +10236,7 @@
         <v>445</v>
       </c>
       <c r="D106" s="52">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E106" s="52">
         <v>8</v>
@@ -10292,7 +10244,7 @@
       <c r="F106" s="52">
         <v>8</v>
       </c>
-      <c r="G106" s="74">
+      <c r="G106" s="52">
         <v>6</v>
       </c>
     </row>
@@ -10304,7 +10256,7 @@
         <v>445</v>
       </c>
       <c r="D107" s="52">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E107" s="52">
         <v>9</v>
@@ -10312,7 +10264,7 @@
       <c r="F107" s="52">
         <v>9</v>
       </c>
-      <c r="G107" s="74">
+      <c r="G107" s="52">
         <v>10</v>
       </c>
     </row>
@@ -10324,7 +10276,7 @@
         <v>445</v>
       </c>
       <c r="D108" s="52">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E108" s="52">
         <v>10</v>
@@ -10332,7 +10284,7 @@
       <c r="F108" s="52">
         <v>10</v>
       </c>
-      <c r="G108" s="74">
+      <c r="G108" s="52">
         <v>2</v>
       </c>
     </row>
@@ -10344,7 +10296,7 @@
         <v>452</v>
       </c>
       <c r="D109" s="52">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E109" s="52">
         <v>2</v>
@@ -10352,7 +10304,7 @@
       <c r="F109" s="52">
         <v>2</v>
       </c>
-      <c r="G109" s="74">
+      <c r="G109" s="52">
         <v>9</v>
       </c>
     </row>
@@ -10364,7 +10316,7 @@
         <v>453</v>
       </c>
       <c r="D110" s="52">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E110" s="52">
         <v>4</v>
@@ -10372,7 +10324,7 @@
       <c r="F110" s="52">
         <v>4</v>
       </c>
-      <c r="G110" s="74">
+      <c r="G110" s="52">
         <v>5</v>
       </c>
     </row>
@@ -10384,7 +10336,7 @@
         <v>454</v>
       </c>
       <c r="D111" s="52">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E111" s="52">
         <v>6</v>
@@ -10392,7 +10344,7 @@
       <c r="F111" s="52">
         <v>6</v>
       </c>
-      <c r="G111" s="74">
+      <c r="G111" s="52">
         <v>1</v>
       </c>
     </row>
@@ -10400,13 +10352,13 @@
     <row r="113" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="114" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="49" t="s">
-        <v>535</v>
-      </c>
-      <c r="B114" s="48" t="s">
+        <v>523</v>
+      </c>
+      <c r="B114" s="62" t="s">
         <v>300</v>
       </c>
       <c r="E114" s="49" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="115" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10427,35 +10379,35 @@
       </c>
     </row>
     <row r="116" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B116" s="69" t="s">
-        <v>550</v>
-      </c>
-      <c r="C116" s="70"/>
-      <c r="D116" s="70"/>
-      <c r="E116" s="70"/>
-      <c r="F116" s="70"/>
+      <c r="B116" s="75" t="s">
+        <v>538</v>
+      </c>
+      <c r="C116" s="76"/>
+      <c r="D116" s="76"/>
+      <c r="E116" s="76"/>
+      <c r="F116" s="76"/>
     </row>
     <row r="117" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B117" s="71"/>
-      <c r="C117" s="71"/>
-      <c r="D117" s="71"/>
-      <c r="E117" s="71"/>
-      <c r="F117" s="71"/>
+      <c r="B117" s="73"/>
+      <c r="C117" s="73"/>
+      <c r="D117" s="73"/>
+      <c r="E117" s="73"/>
+      <c r="F117" s="73"/>
     </row>
     <row r="118" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B118" s="71"/>
-      <c r="C118" s="71"/>
-      <c r="D118" s="71"/>
-      <c r="E118" s="71"/>
-      <c r="F118" s="71"/>
+      <c r="B118" s="73"/>
+      <c r="C118" s="73"/>
+      <c r="D118" s="73"/>
+      <c r="E118" s="73"/>
+      <c r="F118" s="73"/>
     </row>
     <row r="119" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="120" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="121" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="49" t="s">
-        <v>534</v>
-      </c>
-      <c r="B121" s="48" t="s">
+        <v>522</v>
+      </c>
+      <c r="B121" s="62" t="s">
         <v>278</v>
       </c>
     </row>
@@ -10480,7 +10432,7 @@
         <v>2</v>
       </c>
       <c r="C124" s="52" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="125" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10496,16 +10448,16 @@
         <v>4</v>
       </c>
       <c r="C126" s="52" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="127" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="128" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="129" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="49" t="s">
-        <v>534</v>
-      </c>
-      <c r="B129" s="48" t="s">
+        <v>522</v>
+      </c>
+      <c r="B129" s="62" t="s">
         <v>282</v>
       </c>
     </row>
@@ -10514,39 +10466,43 @@
         <v>283</v>
       </c>
       <c r="C130" s="41" t="s">
-        <v>284</v>
+        <v>560</v>
       </c>
       <c r="D130" s="2" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="131" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B131" s="66" t="s">
-        <v>461</v>
-      </c>
-      <c r="C131" s="67"/>
-      <c r="D131" s="68"/>
+      <c r="B131" s="52">
+        <v>1</v>
+      </c>
+      <c r="C131" s="52">
+        <v>1</v>
+      </c>
+      <c r="D131" s="52">
+        <v>2</v>
+      </c>
     </row>
     <row r="132" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B132" s="52">
         <v>1</v>
       </c>
       <c r="C132" s="52">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D132" s="52">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="133" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B133" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C133" s="52">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D133" s="52">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="134" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10554,7 +10510,7 @@
         <v>2</v>
       </c>
       <c r="C134" s="52">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D134" s="52">
         <v>2</v>
@@ -10562,13 +10518,13 @@
     </row>
     <row r="135" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B135" s="52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C135" s="52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D135" s="52">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="136" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10576,7 +10532,7 @@
         <v>3</v>
       </c>
       <c r="C136" s="52">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D136" s="52">
         <v>4</v>
@@ -10584,13 +10540,13 @@
     </row>
     <row r="137" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B137" s="52">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C137" s="52">
+        <v>8</v>
+      </c>
+      <c r="D137" s="52">
         <v>2</v>
-      </c>
-      <c r="D137" s="52">
-        <v>4</v>
       </c>
     </row>
     <row r="138" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10598,21 +10554,21 @@
         <v>4</v>
       </c>
       <c r="C138" s="52">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D138" s="52">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="139" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B139" s="52">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C139" s="52">
-        <v>12</v>
+        <v>88</v>
       </c>
       <c r="D139" s="52">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10620,10 +10576,10 @@
         <v>5</v>
       </c>
       <c r="C140" s="52">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="D140" s="52">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="141" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10631,10 +10587,10 @@
         <v>5</v>
       </c>
       <c r="C141" s="52">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D141" s="52">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10642,7 +10598,7 @@
         <v>5</v>
       </c>
       <c r="C142" s="52">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D142" s="52">
         <v>1</v>
@@ -10650,10 +10606,10 @@
     </row>
     <row r="143" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B143" s="52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C143" s="52">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="D143" s="52">
         <v>1</v>
@@ -10661,24 +10617,24 @@
     </row>
     <row r="144" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B144" s="52">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C144" s="52">
+        <v>1</v>
+      </c>
+      <c r="D144" s="52">
         <v>2</v>
-      </c>
-      <c r="D144" s="52">
-        <v>1</v>
       </c>
     </row>
     <row r="145" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B145" s="52">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C145" s="52">
+        <v>27</v>
+      </c>
+      <c r="D145" s="52">
         <v>1</v>
-      </c>
-      <c r="D145" s="52">
-        <v>2</v>
       </c>
     </row>
     <row r="146" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10686,7 +10642,7 @@
         <v>8</v>
       </c>
       <c r="C146" s="52">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D146" s="52">
         <v>1</v>
@@ -10697,21 +10653,21 @@
         <v>8</v>
       </c>
       <c r="C147" s="52">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="D147" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B148" s="52">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C148" s="52">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D148" s="52">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="149" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10719,10 +10675,10 @@
         <v>9</v>
       </c>
       <c r="C149" s="52">
-        <v>100</v>
+        <v>11</v>
       </c>
       <c r="D149" s="52">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="150" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10730,10 +10686,10 @@
         <v>9</v>
       </c>
       <c r="C150" s="52">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="D150" s="52">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="151" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10741,7 +10697,7 @@
         <v>9</v>
       </c>
       <c r="C151" s="52">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="D151" s="52">
         <v>2</v>
@@ -10752,21 +10708,21 @@
         <v>9</v>
       </c>
       <c r="C152" s="52">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="D152" s="52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="153" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B153" s="52">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C153" s="52">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D153" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="154" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10774,21 +10730,21 @@
         <v>10</v>
       </c>
       <c r="C154" s="52">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="D154" s="52">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="155" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B155" s="52">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C155" s="52">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D155" s="52">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="156" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10796,10 +10752,10 @@
         <v>11</v>
       </c>
       <c r="C156" s="52">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="D156" s="52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="157" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10807,7 +10763,7 @@
         <v>11</v>
       </c>
       <c r="C157" s="52">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="D157" s="52">
         <v>1</v>
@@ -10818,10 +10774,10 @@
         <v>11</v>
       </c>
       <c r="C158" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D158" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="159" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10829,10 +10785,10 @@
         <v>11</v>
       </c>
       <c r="C159" s="52">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D159" s="52">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="160" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10840,29 +10796,29 @@
         <v>11</v>
       </c>
       <c r="C160" s="52">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D160" s="52">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="161" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B161" s="52">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C161" s="52">
-        <v>7</v>
+        <v>55</v>
       </c>
       <c r="D161" s="52">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="162" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B162" s="52">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C162" s="52">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="D162" s="52">
         <v>1</v>
@@ -10873,119 +10829,120 @@
         <v>13</v>
       </c>
       <c r="C163" s="52">
-        <v>92</v>
+        <v>14</v>
       </c>
       <c r="D163" s="52">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="49" t="s">
+        <v>522</v>
+      </c>
+      <c r="B166" s="62" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B167" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B168" s="52">
         <v>1</v>
       </c>
-    </row>
-    <row r="164" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B164" s="52">
-        <v>13</v>
-      </c>
-      <c r="C164" s="52">
-        <v>14</v>
-      </c>
-      <c r="D164" s="52">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A167" s="49" t="s">
-        <v>534</v>
-      </c>
-      <c r="B167" s="48" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B168" s="11" t="s">
-        <v>288</v>
-      </c>
-      <c r="C168" s="2" t="s">
-        <v>289</v>
+      <c r="C168" s="52" t="s">
+        <v>460</v>
       </c>
     </row>
     <row r="169" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B169" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C169" s="52" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="170" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B170" s="52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C170" s="52" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="171" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B171" s="52">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C171" s="52" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="172" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B172" s="52">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C172" s="52" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="173" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B173" s="52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C173" s="52" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="174" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B174" s="52">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C174" s="52" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="49" t="s">
+        <v>523</v>
+      </c>
+      <c r="B177" s="62" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="178" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B178" s="41" t="s">
+        <v>293</v>
+      </c>
+      <c r="C178" s="41" t="s">
+        <v>294</v>
+      </c>
+      <c r="D178" s="40" t="s">
+        <v>295</v>
+      </c>
+      <c r="E178" s="2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="179" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B179" s="57" t="s">
         <v>467</v>
       </c>
-    </row>
-    <row r="175" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B175" s="52">
-        <v>7</v>
-      </c>
-      <c r="C175" s="52" t="s">
+      <c r="C179" s="49"/>
+      <c r="D179" s="49" t="s">
         <v>468</v>
       </c>
-    </row>
-    <row r="176" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A178" s="49" t="s">
-        <v>535</v>
-      </c>
-      <c r="B178" s="48" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="179" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B179" s="41" t="s">
-        <v>293</v>
-      </c>
-      <c r="C179" s="41" t="s">
-        <v>294</v>
-      </c>
-      <c r="D179" s="40" t="s">
-        <v>295</v>
-      </c>
-      <c r="E179" s="2" t="s">
-        <v>296</v>
+      <c r="E179" s="44" t="s">
+        <v>540</v>
       </c>
     </row>
     <row r="180" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -10996,20 +10953,20 @@
       <c r="D180" s="49" t="s">
         <v>470</v>
       </c>
-      <c r="E180" s="44" t="s">
-        <v>552</v>
+      <c r="E180" s="58" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="181" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B181" s="57" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C181" s="49"/>
       <c r="D181" s="49" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E181" s="58" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="182" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -11021,389 +10978,403 @@
         <v>475</v>
       </c>
       <c r="E182" s="58" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="183" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B183" s="57" t="s">
-        <v>476</v>
+        <v>539</v>
       </c>
       <c r="C183" s="49"/>
       <c r="D183" s="49" t="s">
-        <v>477</v>
-      </c>
-      <c r="E183" s="58" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="184" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B184" s="57" t="s">
-        <v>551</v>
-      </c>
-      <c r="C184" s="49"/>
-      <c r="D184" s="49" t="s">
-        <v>478</v>
-      </c>
-      <c r="E184" s="49"/>
-    </row>
+        <v>476</v>
+      </c>
+      <c r="E183" s="49"/>
+    </row>
+    <row r="184" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="185" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="186" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="49" t="s">
+        <v>522</v>
+      </c>
+      <c r="B187" s="62" t="s">
+        <v>306</v>
+      </c>
+    </row>
     <row r="188" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A188" s="49" t="s">
-        <v>534</v>
-      </c>
-      <c r="B188" s="48" t="s">
-        <v>306</v>
+      <c r="B188" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="C188" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D188" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="E188" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="F188" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="G188" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="H188" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="J188" s="62" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="189" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B189" s="11" t="s">
-        <v>307</v>
-      </c>
-      <c r="C189" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D189" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="E189" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="F189" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="G189" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="H189" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="J189" s="62" t="s">
-        <v>322</v>
+      <c r="B189" s="52">
+        <v>1</v>
+      </c>
+      <c r="C189" s="52" t="s">
+        <v>549</v>
+      </c>
+      <c r="D189" s="56" t="s">
+        <v>477</v>
+      </c>
+      <c r="E189" s="52" t="s">
+        <v>438</v>
+      </c>
+      <c r="F189" s="52">
+        <v>123456789</v>
+      </c>
+      <c r="G189" s="59" t="s">
+        <v>479</v>
+      </c>
+      <c r="H189" s="52" t="s">
+        <v>478</v>
+      </c>
+      <c r="J189" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="K189" s="11" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="190" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B190" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C190" s="52" t="s">
-        <v>479</v>
-      </c>
-      <c r="D190" s="56" t="s">
+        <v>550</v>
+      </c>
+      <c r="D190" s="52" t="s">
         <v>480</v>
       </c>
       <c r="E190" s="52" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="F190" s="52">
         <v>123456789</v>
       </c>
       <c r="G190" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H190" s="52" t="s">
         <v>481</v>
       </c>
-      <c r="J190" s="11" t="s">
-        <v>323</v>
-      </c>
-      <c r="K190" s="11" t="s">
-        <v>324</v>
+      <c r="J190" s="52">
+        <v>1</v>
+      </c>
+      <c r="K190" s="52" t="s">
+        <v>520</v>
       </c>
     </row>
     <row r="191" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B191" s="52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C191" s="52" t="s">
-        <v>483</v>
+        <v>551</v>
       </c>
       <c r="D191" s="52" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="E191" s="52" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F191" s="52">
         <v>123456789</v>
       </c>
       <c r="G191" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H191" s="52" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="J191" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K191" s="52" t="s">
-        <v>532</v>
+        <v>519</v>
       </c>
     </row>
     <row r="192" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B192" s="52">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C192" s="52" t="s">
-        <v>486</v>
+        <v>552</v>
       </c>
       <c r="D192" s="52" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="E192" s="52" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="F192" s="52">
         <v>123456789</v>
       </c>
       <c r="G192" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H192" s="52" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="J192" s="52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K192" s="52" t="s">
-        <v>531</v>
+        <v>518</v>
       </c>
     </row>
     <row r="193" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B193" s="52">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C193" s="52" t="s">
-        <v>489</v>
+        <v>553</v>
       </c>
       <c r="D193" s="52" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="E193" s="52" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F193" s="52">
         <v>123456789</v>
       </c>
       <c r="G193" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H193" s="52" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="J193" s="52">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K193" s="52" t="s">
-        <v>530</v>
+        <v>517</v>
       </c>
     </row>
     <row r="194" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B194" s="52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C194" s="52" t="s">
-        <v>492</v>
+        <v>554</v>
       </c>
       <c r="D194" s="52" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
       <c r="E194" s="52" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F194" s="52">
         <v>123456789</v>
       </c>
       <c r="G194" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H194" s="52" t="s">
-        <v>494</v>
-      </c>
-      <c r="J194" s="52">
-        <v>4</v>
-      </c>
-      <c r="K194" s="52" t="s">
-        <v>529</v>
+        <v>489</v>
       </c>
     </row>
     <row r="195" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B195" s="52">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C195" s="52" t="s">
-        <v>495</v>
+        <v>555</v>
       </c>
       <c r="D195" s="52" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="E195" s="52" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F195" s="52">
         <v>123456789</v>
       </c>
       <c r="G195" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H195" s="52" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
     </row>
     <row r="196" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B196" s="52">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C196" s="52" t="s">
-        <v>498</v>
+        <v>556</v>
       </c>
       <c r="D196" s="52" t="s">
-        <v>499</v>
+        <v>492</v>
       </c>
       <c r="E196" s="52" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F196" s="52">
         <v>123456789</v>
       </c>
       <c r="G196" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H196" s="52" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
     </row>
     <row r="197" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B197" s="52">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C197" s="52" t="s">
-        <v>501</v>
+        <v>557</v>
       </c>
       <c r="D197" s="52" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="E197" s="52" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F197" s="52">
         <v>123456789</v>
       </c>
       <c r="G197" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H197" s="52" t="s">
-        <v>503</v>
+        <v>495</v>
       </c>
     </row>
     <row r="198" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B198" s="52">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C198" s="52" t="s">
-        <v>504</v>
+        <v>558</v>
       </c>
       <c r="D198" s="52" t="s">
-        <v>505</v>
+        <v>496</v>
       </c>
       <c r="E198" s="52" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="F198" s="52">
         <v>123456789</v>
       </c>
       <c r="G198" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H198" s="52" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="199" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B199" s="52">
-        <v>10</v>
-      </c>
-      <c r="C199" s="52" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="199" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I200" s="49" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="201" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B201" s="62" t="s">
+        <v>314</v>
+      </c>
+      <c r="I201" s="61" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="202" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B202" s="11" t="s">
+        <v>315</v>
+      </c>
+      <c r="C202" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="D202" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="E202" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="F202" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="G202" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="H202" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="I202" s="40" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="203" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B203" s="52">
+        <v>1</v>
+      </c>
+      <c r="C203" s="52" t="s">
+        <v>468</v>
+      </c>
+      <c r="D203" s="56" t="s">
+        <v>535</v>
+      </c>
+      <c r="E203" s="52" t="s">
+        <v>438</v>
+      </c>
+      <c r="F203" s="52">
+        <v>123456789</v>
+      </c>
+      <c r="G203" s="59" t="s">
+        <v>479</v>
+      </c>
+      <c r="H203" s="52" t="s">
         <v>507</v>
       </c>
-      <c r="D199" s="52" t="s">
-        <v>508</v>
-      </c>
-      <c r="E199" s="52" t="s">
-        <v>451</v>
-      </c>
-      <c r="F199" s="52">
-        <v>123456789</v>
-      </c>
-      <c r="G199" s="59" t="s">
-        <v>482</v>
-      </c>
-      <c r="H199" s="52" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="200" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I201" s="49" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="202" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B202" s="62" t="s">
-        <v>314</v>
-      </c>
-      <c r="I202" s="61" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="203" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B203" s="11" t="s">
-        <v>315</v>
-      </c>
-      <c r="C203" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="D203" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="E203" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="F203" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="G203" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="H203" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="I203" s="40" t="s">
-        <v>325</v>
+      <c r="I203" s="52">
+        <v>1</v>
       </c>
     </row>
     <row r="204" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B204" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C204" s="52" t="s">
-        <v>470</v>
-      </c>
-      <c r="D204" s="56" t="s">
-        <v>547</v>
+        <v>506</v>
+      </c>
+      <c r="D204" s="49" t="s">
+        <v>536</v>
       </c>
       <c r="E204" s="52" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="F204" s="52">
         <v>123456789</v>
       </c>
       <c r="G204" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H204" s="52" t="s">
-        <v>519</v>
+        <v>508</v>
       </c>
       <c r="I204" s="52">
         <v>1</v>
@@ -11411,77 +11382,77 @@
     </row>
     <row r="205" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B205" s="52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C205" s="52" t="s">
-        <v>518</v>
-      </c>
-      <c r="D205" s="49" t="s">
-        <v>548</v>
+        <v>505</v>
+      </c>
+      <c r="D205" s="56" t="s">
+        <v>535</v>
       </c>
       <c r="E205" s="52" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F205" s="52">
         <v>123456789</v>
       </c>
       <c r="G205" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H205" s="52" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
       <c r="I205" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="206" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B206" s="52">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C206" s="52" t="s">
-        <v>517</v>
-      </c>
-      <c r="D206" s="56" t="s">
-        <v>547</v>
+        <v>504</v>
+      </c>
+      <c r="D206" s="49" t="s">
+        <v>536</v>
       </c>
       <c r="E206" s="52" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="F206" s="52">
         <v>123456789</v>
       </c>
       <c r="G206" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H206" s="52" t="s">
-        <v>521</v>
+        <v>510</v>
       </c>
       <c r="I206" s="52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B207" s="52">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C207" s="52" t="s">
-        <v>516</v>
-      </c>
-      <c r="D207" s="49" t="s">
-        <v>548</v>
+        <v>503</v>
+      </c>
+      <c r="D207" s="56" t="s">
+        <v>535</v>
       </c>
       <c r="E207" s="52" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F207" s="52">
         <v>123456789</v>
       </c>
       <c r="G207" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H207" s="52" t="s">
-        <v>522</v>
+        <v>511</v>
       </c>
       <c r="I207" s="52">
         <v>1</v>
@@ -11489,25 +11460,25 @@
     </row>
     <row r="208" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B208" s="52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C208" s="52" t="s">
-        <v>515</v>
-      </c>
-      <c r="D208" s="56" t="s">
-        <v>547</v>
+        <v>502</v>
+      </c>
+      <c r="D208" s="49" t="s">
+        <v>536</v>
       </c>
       <c r="E208" s="52" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F208" s="52">
         <v>123456789</v>
       </c>
       <c r="G208" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H208" s="52" t="s">
-        <v>523</v>
+        <v>512</v>
       </c>
       <c r="I208" s="52">
         <v>1</v>
@@ -11515,315 +11486,300 @@
     </row>
     <row r="209" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B209" s="52">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C209" s="52" t="s">
-        <v>514</v>
-      </c>
-      <c r="D209" s="49" t="s">
-        <v>548</v>
+        <v>501</v>
+      </c>
+      <c r="D209" s="56" t="s">
+        <v>535</v>
       </c>
       <c r="E209" s="52" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F209" s="52">
         <v>123456789</v>
       </c>
       <c r="G209" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H209" s="52" t="s">
-        <v>524</v>
+        <v>513</v>
       </c>
       <c r="I209" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="210" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B210" s="52">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C210" s="52" t="s">
-        <v>513</v>
-      </c>
-      <c r="D210" s="56" t="s">
-        <v>547</v>
+        <v>500</v>
+      </c>
+      <c r="D210" s="49" t="s">
+        <v>536</v>
       </c>
       <c r="E210" s="52" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F210" s="52">
         <v>123456789</v>
       </c>
       <c r="G210" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H210" s="52" t="s">
-        <v>525</v>
+        <v>514</v>
       </c>
       <c r="I210" s="52">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="211" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B211" s="52">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C211" s="52" t="s">
-        <v>512</v>
-      </c>
-      <c r="D211" s="49" t="s">
-        <v>548</v>
+        <v>499</v>
+      </c>
+      <c r="D211" s="56" t="s">
+        <v>535</v>
       </c>
       <c r="E211" s="52" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F211" s="52">
         <v>123456789</v>
       </c>
       <c r="G211" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H211" s="52" t="s">
-        <v>526</v>
+        <v>515</v>
       </c>
       <c r="I211" s="52">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="212" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B212" s="52">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C212" s="52" t="s">
-        <v>511</v>
-      </c>
-      <c r="D212" s="56" t="s">
-        <v>547</v>
+        <v>498</v>
+      </c>
+      <c r="D212" s="49" t="s">
+        <v>536</v>
       </c>
       <c r="E212" s="52" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="F212" s="52">
         <v>123456789</v>
       </c>
       <c r="G212" s="59" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="H212" s="52" t="s">
-        <v>527</v>
+        <v>516</v>
       </c>
       <c r="I212" s="52">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="214" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="215" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A215" s="49" t="s">
+        <v>523</v>
+      </c>
+      <c r="B215" s="62" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="216" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B216" s="11" t="s">
+        <v>327</v>
+      </c>
+      <c r="C216" s="40" t="s">
+        <v>328</v>
+      </c>
+      <c r="D216" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="E216" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="F216" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="217" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B217" s="69" t="s">
+        <v>542</v>
+      </c>
+      <c r="C217" s="70"/>
+      <c r="D217" s="70"/>
+      <c r="E217" s="70"/>
+      <c r="F217" s="70"/>
+    </row>
+    <row r="218" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B218" s="71"/>
+      <c r="C218" s="71"/>
+      <c r="D218" s="71"/>
+      <c r="E218" s="71"/>
+      <c r="F218" s="71"/>
+    </row>
+    <row r="219" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B219" s="71"/>
+      <c r="C219" s="71"/>
+      <c r="D219" s="71"/>
+      <c r="E219" s="71"/>
+      <c r="F219" s="71"/>
+    </row>
+    <row r="220" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="221" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="222" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A222" s="49" t="s">
+        <v>522</v>
+      </c>
+      <c r="B222" s="62" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="223" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B223" s="11" t="s">
+        <v>333</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="D223" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="E223" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="F223" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="G223" s="2" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="224" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B224" s="66" t="s">
+        <v>543</v>
+      </c>
+      <c r="C224" s="67"/>
+      <c r="D224" s="67"/>
+      <c r="E224" s="67"/>
+      <c r="F224" s="67"/>
+      <c r="G224" s="67"/>
+    </row>
+    <row r="225" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B225" s="68"/>
+      <c r="C225" s="68"/>
+      <c r="D225" s="68"/>
+      <c r="E225" s="68"/>
+      <c r="F225" s="68"/>
+      <c r="G225" s="68"/>
+    </row>
+    <row r="226" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="227" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="228" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A228" s="49" t="s">
+        <v>522</v>
+      </c>
+      <c r="B228" s="60" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B229" s="11" t="s">
+        <v>340</v>
+      </c>
+      <c r="C229" s="38" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B230" s="52">
         <v>1</v>
       </c>
-    </row>
-    <row r="213" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B213" s="52">
-        <v>10</v>
-      </c>
-      <c r="C213" s="52" t="s">
-        <v>510</v>
-      </c>
-      <c r="D213" s="49" t="s">
-        <v>548</v>
-      </c>
-      <c r="E213" s="52" t="s">
-        <v>451</v>
-      </c>
-      <c r="F213" s="52">
-        <v>123456789</v>
-      </c>
-      <c r="G213" s="59" t="s">
-        <v>482</v>
-      </c>
-      <c r="H213" s="52" t="s">
-        <v>528</v>
-      </c>
-      <c r="I213" s="52">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="214" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="215" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="216" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B216" s="48" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="217" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B217" s="11" t="s">
-        <v>327</v>
-      </c>
-      <c r="C217" s="40" t="s">
-        <v>328</v>
-      </c>
-      <c r="D217" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="E217" s="2" t="s">
-        <v>553</v>
-      </c>
-      <c r="F217" s="2" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="218" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B218" s="75" t="s">
-        <v>554</v>
-      </c>
-      <c r="C218" s="76"/>
-      <c r="D218" s="76"/>
-      <c r="E218" s="76"/>
-      <c r="F218" s="76"/>
-    </row>
-    <row r="219" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B219" s="77"/>
-      <c r="C219" s="77"/>
-      <c r="D219" s="77"/>
-      <c r="E219" s="77"/>
-      <c r="F219" s="77"/>
-    </row>
-    <row r="220" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B220" s="77"/>
-      <c r="C220" s="77"/>
-      <c r="D220" s="77"/>
-      <c r="E220" s="77"/>
-      <c r="F220" s="77"/>
-    </row>
-    <row r="221" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A223" s="49" t="s">
-        <v>534</v>
-      </c>
-      <c r="B223" s="48" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="224" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B224" s="11" t="s">
-        <v>333</v>
-      </c>
-      <c r="C224" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="D224" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="E224" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="F224" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="G224" s="2" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="225" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B225" s="80" t="s">
-        <v>555</v>
-      </c>
-      <c r="C225" s="79"/>
-      <c r="D225" s="79"/>
-      <c r="E225" s="79"/>
-      <c r="F225" s="79"/>
-      <c r="G225" s="79"/>
-    </row>
-    <row r="226" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B226" s="78"/>
-      <c r="C226" s="78"/>
-      <c r="D226" s="78"/>
-      <c r="E226" s="78"/>
-      <c r="F226" s="78"/>
-      <c r="G226" s="78"/>
-    </row>
-    <row r="227" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A229" s="49" t="s">
-        <v>534</v>
-      </c>
-      <c r="B229" s="60" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="230" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B230" s="11" t="s">
-        <v>340</v>
-      </c>
-      <c r="C230" s="38" t="s">
-        <v>341</v>
+      <c r="C230" s="52" t="s">
+        <v>544</v>
       </c>
     </row>
     <row r="231" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B231" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C231" s="52" t="s">
-        <v>556</v>
+        <v>545</v>
       </c>
     </row>
     <row r="232" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B232" s="52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C232" s="52" t="s">
-        <v>557</v>
+        <v>546</v>
       </c>
     </row>
     <row r="233" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B233" s="52">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C233" s="52" t="s">
-        <v>558</v>
+        <v>547</v>
       </c>
     </row>
     <row r="234" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B234" s="52">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C234" s="52" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="235" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B235" s="52">
-        <v>5</v>
-      </c>
-      <c r="C235" s="52" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="236" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>548</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="236" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A236" s="49" t="s">
+        <v>522</v>
+      </c>
+      <c r="B236" s="48" t="s">
+        <v>342</v>
+      </c>
+    </row>
     <row r="237" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A237" s="49" t="s">
-        <v>534</v>
-      </c>
-      <c r="B237" s="48" t="s">
-        <v>342</v>
+      <c r="B237" s="41" t="s">
+        <v>343</v>
+      </c>
+      <c r="C237" s="41" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="238" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B238" s="41" t="s">
-        <v>343</v>
-      </c>
-      <c r="C238" s="41" t="s">
-        <v>374</v>
+      <c r="B238" s="52">
+        <v>1</v>
+      </c>
+      <c r="C238" s="52">
+        <v>1</v>
       </c>
     </row>
     <row r="239" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B239" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C239" s="52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="240" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B240" s="52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C240" s="52">
         <v>2</v>
@@ -11831,15 +11787,15 @@
     </row>
     <row r="241" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B241" s="52">
+        <v>4</v>
+      </c>
+      <c r="C241" s="52">
         <v>3</v>
-      </c>
-      <c r="C241" s="52">
-        <v>2</v>
       </c>
     </row>
     <row r="242" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B242" s="52">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C242" s="52">
         <v>3</v>
@@ -11847,15 +11803,15 @@
     </row>
     <row r="243" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B243" s="52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C243" s="52">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="244" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B244" s="52">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C244" s="52">
         <v>4</v>
@@ -11863,15 +11819,15 @@
     </row>
     <row r="245" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B245" s="52">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C245" s="52">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="246" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B246" s="52">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C246" s="52">
         <v>5</v>
@@ -11879,20 +11835,13 @@
     </row>
     <row r="247" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B247" s="52">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C247" s="52">
         <v>5</v>
       </c>
     </row>
-    <row r="248" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B248" s="52">
-        <v>10</v>
-      </c>
-      <c r="C248" s="52">
-        <v>5</v>
-      </c>
-    </row>
+    <row r="248" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="249" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="250" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="251" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -12644,12 +12593,10 @@
     <row r="997" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="998" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="999" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="1000" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B225:G226"/>
-    <mergeCell ref="B131:D131"/>
-    <mergeCell ref="B218:F220"/>
+  <mergeCells count="7">
+    <mergeCell ref="B224:G225"/>
+    <mergeCell ref="B217:F219"/>
     <mergeCell ref="C43:F46"/>
     <mergeCell ref="C51:C60"/>
     <mergeCell ref="C65:F68"/>

</xml_diff>